<commit_message>
improved existing plots, added plots for standard metric both sorted by energy and grouped by alpha/depth
</commit_message>
<xml_diff>
--- a/results/plots/grid_analysis/grid_budget_tables.xlsx
+++ b/results/plots/grid_analysis/grid_budget_tables.xlsx
@@ -7,25 +7,31 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="A0.25_D04" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="A0.25_D06" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="A0.25_D08" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="A0.25_D10" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="A0.75_D02" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="A0.75_D04" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="A0.75_D06" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="A0.75_D08" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="A0.75_D10" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="A1.0_D02" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="A1.0_D04" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="A1.0_D06" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="A1.0_D08" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="A1.0_D10" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="A1.25_D02" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="A1.25_D04" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="A1.25_D06" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="A1.25_D08" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="A1.25_D10" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="A0.25_D02" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="A0.25_D04" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="A0.25_D06" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="A0.25_D08" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="A0.25_D10" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="A0.5_D02" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="A0.5_D04" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="A0.5_D06" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="A0.5_D08" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="A0.5_D10" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="A0.75_D02" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="A0.75_D04" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="A0.75_D06" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="A0.75_D08" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="A0.75_D10" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="A1.0_D02" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="A1.0_D04" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="A1.0_D06" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="A1.0_D08" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="A1.0_D10" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="A1.25_D02" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="A1.25_D04" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="A1.25_D06" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="A1.25_D08" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="A1.25_D10" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,27 +487,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -513,27 +519,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>53 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>53 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>53 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>53 (E)</t>
         </is>
       </c>
     </row>
@@ -545,27 +551,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>173 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>346 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>535 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>535 (E)</t>
         </is>
       </c>
     </row>
@@ -577,27 +583,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>173 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>346 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9 (T)</t>
+          <t>1039 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>18 (T)</t>
+          <t>2078 (T)</t>
         </is>
       </c>
     </row>
@@ -650,27 +656,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -682,27 +688,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
     </row>
@@ -714,27 +720,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>542 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>542 (E)</t>
         </is>
       </c>
     </row>
@@ -746,27 +752,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12 (T)</t>
+          <t>1076 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>24 (T)</t>
+          <t>2152 (T)</t>
         </is>
       </c>
     </row>
@@ -819,27 +825,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -851,27 +857,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>43 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
     </row>
@@ -883,27 +889,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>43 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>215 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>430 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>623 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>623 (E)</t>
         </is>
       </c>
     </row>
@@ -915,27 +921,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>43 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>215 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>430 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13 (T)</t>
+          <t>1292 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>27 (T)</t>
+          <t>2585 (T)</t>
         </is>
       </c>
     </row>
@@ -988,27 +994,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -1020,27 +1026,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
     </row>
@@ -1052,27 +1058,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>606 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>606 (E)</t>
         </is>
       </c>
     </row>
@@ -1084,27 +1090,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11 (T)</t>
+          <t>1244 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>23 (T)</t>
+          <t>2488 (T)</t>
         </is>
       </c>
     </row>
@@ -1157,27 +1163,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -1189,27 +1195,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>39 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
     </row>
@@ -1221,27 +1227,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>39 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>198 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>396 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>560 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>560 (E)</t>
         </is>
       </c>
     </row>
@@ -1253,27 +1259,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>39 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>198 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>396 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10 (T)</t>
+          <t>1188 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>21 (T)</t>
+          <t>2377 (T)</t>
         </is>
       </c>
     </row>
@@ -1326,27 +1332,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -1358,27 +1364,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
     </row>
@@ -1390,27 +1396,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>191 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>383 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>519 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>519 (E)</t>
         </is>
       </c>
     </row>
@@ -1422,27 +1428,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>191 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>383 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10 (T)</t>
+          <t>1151 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>20 (T)</t>
+          <t>2303 (T)</t>
         </is>
       </c>
     </row>
@@ -1495,27 +1501,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -1527,27 +1533,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
     </row>
@@ -1559,27 +1565,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>491 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>491 (E)</t>
         </is>
       </c>
     </row>
@@ -1591,27 +1597,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12 (T)</t>
+          <t>1074 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>24 (T)</t>
+          <t>2148 (T)</t>
         </is>
       </c>
     </row>
@@ -1664,27 +1670,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -1696,27 +1702,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
     </row>
@@ -1728,27 +1734,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>581 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>581 (E)</t>
         </is>
       </c>
     </row>
@@ -1760,27 +1766,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11 (T)</t>
+          <t>1242 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>23 (T)</t>
+          <t>2484 (T)</t>
         </is>
       </c>
     </row>
@@ -1833,27 +1839,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -1865,27 +1871,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>46 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
     </row>
@@ -1897,27 +1903,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>46 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>233 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>466 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>665 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>665 (E)</t>
         </is>
       </c>
     </row>
@@ -1929,27 +1935,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>46 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>233 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>466 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11 (T)</t>
+          <t>1398 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>22 (E)</t>
+          <t>2797 (T)</t>
         </is>
       </c>
     </row>
@@ -2002,27 +2008,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -2034,27 +2040,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
     </row>
@@ -2066,27 +2072,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>500 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>500 (E)</t>
         </is>
       </c>
     </row>
@@ -2098,27 +2104,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10 (T)</t>
+          <t>1158 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>20 (E)</t>
+          <t>2317 (T)</t>
         </is>
       </c>
     </row>
@@ -2171,27 +2177,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -2203,27 +2209,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>36 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
     </row>
@@ -2235,27 +2241,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>36 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>181 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>362 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1 (E)</t>
+          <t>471 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 (E)</t>
+          <t>471 (E)</t>
         </is>
       </c>
     </row>
@@ -2267,27 +2273,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>36 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>181 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>362 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>1086 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7 (T)</t>
+          <t>2173 (T)</t>
         </is>
       </c>
     </row>
@@ -2340,27 +2346,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -2372,27 +2378,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>31 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
     </row>
@@ -2404,27 +2410,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>31 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>155 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>311 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>493 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>493 (E)</t>
         </is>
       </c>
     </row>
@@ -2436,27 +2442,1041 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>31 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>155 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>311 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10 (T)</t>
+          <t>934 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>20 (T)</t>
+          <t>1868 (T)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>33 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>43 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>43 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>43 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>43 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>33 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>167 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>335 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>433 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>433 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>33 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>167 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>335 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1007 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2015 (T)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>5 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>40 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>52 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>52 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>52 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>52 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>40 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>204 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>409 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>526 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>526 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>40 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>204 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>409 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1229 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2459 (T)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>39 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>39 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>195 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>391 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>485 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>485 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>39 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>195 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>391 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1174 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2349 (T)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>37 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>37 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>187 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>374 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>447 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>447 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>37 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>187 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>374 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1122 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2235 (E)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>34 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>34 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>173 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>347 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>417 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>417 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>34 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>173 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>347 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1043 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2086 (E)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>62 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>125 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>172 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>172 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>62 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>125 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>376 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>753 (T)</t>
         </is>
       </c>
     </row>
@@ -2509,27 +3529,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -2541,27 +3561,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>33 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
     </row>
@@ -2573,27 +3593,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>33 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>167 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>335 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>523 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>523 (E)</t>
         </is>
       </c>
     </row>
@@ -2605,27 +3625,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>33 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>167 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>335 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9 (T)</t>
+          <t>1005 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>19 (T)</t>
+          <t>2011 (T)</t>
         </is>
       </c>
     </row>
@@ -2678,27 +3698,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -2710,27 +3730,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>31 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
     </row>
@@ -2742,27 +3762,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>31 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>158 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>317 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>497 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>497 (E)</t>
         </is>
       </c>
     </row>
@@ -2774,27 +3794,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>31 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>158 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>317 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9 (T)</t>
+          <t>951 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>18 (T)</t>
+          <t>1902 (T)</t>
         </is>
       </c>
     </row>
@@ -2847,27 +3867,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -2879,27 +3899,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>30 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
     </row>
@@ -2911,27 +3931,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>30 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>153 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>306 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12 (T)</t>
+          <t>503 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>24 (E)</t>
+          <t>503 (E)</t>
         </is>
       </c>
     </row>
@@ -2943,27 +3963,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>30 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>153 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>306 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12 (T)</t>
+          <t>920 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>25 (T)</t>
+          <t>1840 (T)</t>
         </is>
       </c>
     </row>
@@ -3016,27 +4036,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -3048,27 +4068,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
     </row>
@@ -3080,27 +4100,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>208 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>417 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>661 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>661 (E)</t>
         </is>
       </c>
     </row>
@@ -3112,27 +4132,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2 (T)</t>
+          <t>208 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4 (T)</t>
+          <t>417 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12 (T)</t>
+          <t>1251 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>24 (T)</t>
+          <t>2502 (T)</t>
         </is>
       </c>
     </row>
@@ -3185,27 +4205,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -3217,27 +4237,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
     </row>
@@ -3249,27 +4269,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>209 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>418 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>658 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>658 (E)</t>
         </is>
       </c>
     </row>
@@ -3281,27 +4301,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>209 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>418 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11 (T)</t>
+          <t>1255 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>23 (T)</t>
+          <t>2511 (T)</t>
         </is>
       </c>
     </row>
@@ -3354,27 +4374,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -3386,27 +4406,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
     </row>
@@ -3418,27 +4438,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>594 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>594 (E)</t>
         </is>
       </c>
     </row>
@@ -3450,27 +4470,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11 (T)</t>
+          <t>1160 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>23 (T)</t>
+          <t>2321 (T)</t>
         </is>
       </c>
     </row>
@@ -3523,27 +4543,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -3555,27 +4575,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
     </row>
@@ -3587,27 +4607,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>190 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>381 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>570 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>570 (E)</t>
         </is>
       </c>
     </row>
@@ -3619,27 +4639,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1 (T)</t>
+          <t>190 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (T)</t>
+          <t>381 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10 (T)</t>
+          <t>1143 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>21 (T)</t>
+          <t>2286 (T)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
coral micro performance plots with depth 12 models
</commit_message>
<xml_diff>
--- a/results/plots/grid_analysis/grid_budget_tables.xlsx
+++ b/results/plots/grid_analysis/grid_budget_tables.xlsx
@@ -12,26 +12,31 @@
     <sheet name="A0.25_D06" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="A0.25_D08" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="A0.25_D10" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="A0.5_D02" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="A0.5_D04" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="A0.5_D06" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="A0.5_D08" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="A0.5_D10" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="A0.75_D02" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="A0.75_D04" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="A0.75_D06" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="A0.75_D08" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="A0.75_D10" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="A1.0_D02" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="A1.0_D04" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="A1.0_D06" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="A1.0_D08" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="A1.0_D10" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="A1.25_D02" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="A1.25_D04" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="A1.25_D06" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="A1.25_D08" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="A1.25_D10" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="A0.25_D12" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="A0.5_D02" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="A0.5_D04" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="A0.5_D06" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="A0.5_D08" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="A0.5_D10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="A0.5_D12" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="A0.75_D02" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="A0.75_D04" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="A0.75_D06" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="A0.75_D08" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="A0.75_D10" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="A0.75_D12" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="A1.0_D02" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="A1.0_D04" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="A1.0_D06" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="A1.0_D08" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="A1.0_D10" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="A1.0_D12" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="A1.25_D02" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="A1.25_D04" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="A1.25_D06" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="A1.25_D08" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="A1.25_D10" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="A1.25_D12" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -688,27 +693,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>54 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>54 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>54 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>54 (E)</t>
+          <t>57 (E)</t>
         </is>
       </c>
     </row>
@@ -720,27 +725,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>179 (T)</t>
+          <t>190 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>358 (T)</t>
+          <t>381 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>542 (E)</t>
+          <t>570 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>542 (E)</t>
+          <t>570 (E)</t>
         </is>
       </c>
     </row>
@@ -752,27 +757,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>179 (T)</t>
+          <t>190 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>358 (T)</t>
+          <t>381 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1076 (T)</t>
+          <t>1143 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2152 (T)</t>
+          <t>2286 (T)</t>
         </is>
       </c>
     </row>
@@ -825,27 +830,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -857,27 +862,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>43 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>62 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>62 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>62 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>62 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
     </row>
@@ -889,27 +894,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>43 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>215 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>430 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>623 (E)</t>
+          <t>542 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>623 (E)</t>
+          <t>542 (E)</t>
         </is>
       </c>
     </row>
@@ -921,27 +926,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>43 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>215 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>430 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1292 (T)</t>
+          <t>1076 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2585 (T)</t>
+          <t>2152 (T)</t>
         </is>
       </c>
     </row>
@@ -994,27 +999,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -1026,27 +1031,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>60 (E)</t>
+          <t>48 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>60 (E)</t>
+          <t>48 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>60 (E)</t>
+          <t>48 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>60 (E)</t>
+          <t>48 (E)</t>
         </is>
       </c>
     </row>
@@ -1058,27 +1063,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>207 (T)</t>
+          <t>173 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>414 (T)</t>
+          <t>347 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>606 (E)</t>
+          <t>489 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>606 (E)</t>
+          <t>489 (E)</t>
         </is>
       </c>
     </row>
@@ -1090,27 +1095,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>207 (T)</t>
+          <t>173 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>414 (T)</t>
+          <t>347 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1244 (T)</t>
+          <t>1043 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2488 (T)</t>
+          <t>2087 (T)</t>
         </is>
       </c>
     </row>
@@ -1163,27 +1168,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -1195,27 +1200,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>39 (T)</t>
+          <t>43 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>56 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>56 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>56 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>56 (E)</t>
+          <t>62 (E)</t>
         </is>
       </c>
     </row>
@@ -1227,27 +1232,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>39 (T)</t>
+          <t>43 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>198 (T)</t>
+          <t>215 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>396 (T)</t>
+          <t>430 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>560 (E)</t>
+          <t>623 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>560 (E)</t>
+          <t>623 (E)</t>
         </is>
       </c>
     </row>
@@ -1259,27 +1264,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>39 (T)</t>
+          <t>43 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>198 (T)</t>
+          <t>215 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>396 (T)</t>
+          <t>430 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1188 (T)</t>
+          <t>1292 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2377 (T)</t>
+          <t>2585 (T)</t>
         </is>
       </c>
     </row>
@@ -1332,27 +1337,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -1364,27 +1369,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>51 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>51 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>51 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>51 (E)</t>
+          <t>60 (E)</t>
         </is>
       </c>
     </row>
@@ -1396,27 +1401,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>191 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>383 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>519 (E)</t>
+          <t>606 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>519 (E)</t>
+          <t>606 (E)</t>
         </is>
       </c>
     </row>
@@ -1428,27 +1433,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>191 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>383 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1151 (T)</t>
+          <t>1244 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2303 (T)</t>
+          <t>2488 (T)</t>
         </is>
       </c>
     </row>
@@ -1501,27 +1506,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -1533,27 +1538,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35 (T)</t>
+          <t>39 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>49 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>49 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>49 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>49 (E)</t>
+          <t>56 (E)</t>
         </is>
       </c>
     </row>
@@ -1565,27 +1570,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35 (T)</t>
+          <t>39 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>179 (T)</t>
+          <t>198 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>358 (T)</t>
+          <t>396 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>491 (E)</t>
+          <t>560 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>491 (E)</t>
+          <t>560 (E)</t>
         </is>
       </c>
     </row>
@@ -1597,27 +1602,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35 (T)</t>
+          <t>39 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>179 (T)</t>
+          <t>198 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>358 (T)</t>
+          <t>396 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1074 (T)</t>
+          <t>1188 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2148 (T)</t>
+          <t>2377 (T)</t>
         </is>
       </c>
     </row>
@@ -1702,27 +1707,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>58 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>58 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>58 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>58 (E)</t>
+          <t>51 (E)</t>
         </is>
       </c>
     </row>
@@ -1734,27 +1739,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>207 (T)</t>
+          <t>191 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>414 (T)</t>
+          <t>383 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>581 (E)</t>
+          <t>519 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>581 (E)</t>
+          <t>519 (E)</t>
         </is>
       </c>
     </row>
@@ -1766,27 +1771,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>207 (T)</t>
+          <t>191 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>414 (T)</t>
+          <t>383 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1242 (T)</t>
+          <t>1151 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2484 (T)</t>
+          <t>2303 (T)</t>
         </is>
       </c>
     </row>
@@ -1839,27 +1844,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -1871,27 +1876,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>46 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>49 (E)</t>
         </is>
       </c>
     </row>
@@ -1903,27 +1908,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>46 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>233 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>466 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>665 (E)</t>
+          <t>491 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>665 (E)</t>
+          <t>491 (E)</t>
         </is>
       </c>
     </row>
@@ -1935,27 +1940,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>46 (T)</t>
+          <t>35 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>233 (T)</t>
+          <t>179 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>466 (T)</t>
+          <t>358 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1398 (T)</t>
+          <t>1074 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2797 (T)</t>
+          <t>2148 (T)</t>
         </is>
       </c>
     </row>
@@ -2008,27 +2013,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -2040,27 +2045,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>50 (E)</t>
+          <t>45 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>50 (E)</t>
+          <t>45 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>50 (E)</t>
+          <t>45 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>50 (E)</t>
+          <t>45 (E)</t>
         </is>
       </c>
     </row>
@@ -2072,27 +2077,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>193 (T)</t>
+          <t>172 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>386 (T)</t>
+          <t>344 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>500 (E)</t>
+          <t>459 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>500 (E)</t>
+          <t>459 (E)</t>
         </is>
       </c>
     </row>
@@ -2104,27 +2109,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>34 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>193 (T)</t>
+          <t>172 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>386 (T)</t>
+          <t>344 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1158 (T)</t>
+          <t>1033 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2317 (T)</t>
+          <t>2066 (T)</t>
         </is>
       </c>
     </row>
@@ -2177,27 +2182,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -2209,27 +2214,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>36 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>47 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>47 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>47 (E)</t>
+          <t>58 (E)</t>
         </is>
       </c>
     </row>
@@ -2241,27 +2246,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>36 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>181 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>362 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>471 (E)</t>
+          <t>581 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>471 (E)</t>
+          <t>581 (E)</t>
         </is>
       </c>
     </row>
@@ -2273,27 +2278,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>36 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>181 (T)</t>
+          <t>207 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>362 (T)</t>
+          <t>414 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1086 (T)</t>
+          <t>1242 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2173 (T)</t>
+          <t>2484 (T)</t>
         </is>
       </c>
     </row>
@@ -2515,27 +2520,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -2547,27 +2552,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>33 (T)</t>
+          <t>40 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>43 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>43 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>43 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>43 (E)</t>
+          <t>54 (E)</t>
         </is>
       </c>
     </row>
@@ -2579,27 +2584,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>33 (T)</t>
+          <t>40 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>167 (T)</t>
+          <t>202 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>335 (T)</t>
+          <t>404 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>433 (E)</t>
+          <t>542 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>433 (E)</t>
+          <t>542 (E)</t>
         </is>
       </c>
     </row>
@@ -2611,27 +2616,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>33 (T)</t>
+          <t>40 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>167 (T)</t>
+          <t>202 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>335 (T)</t>
+          <t>404 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1007 (T)</t>
+          <t>1212 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2015 (T)</t>
+          <t>2424 (T)</t>
         </is>
       </c>
     </row>
@@ -2716,27 +2721,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>40 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>52 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>52 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>52 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>52 (E)</t>
+          <t>50 (E)</t>
         </is>
       </c>
     </row>
@@ -2748,27 +2753,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>40 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>204 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>409 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>526 (E)</t>
+          <t>500 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>526 (E)</t>
+          <t>500 (E)</t>
         </is>
       </c>
     </row>
@@ -2780,27 +2785,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>40 (T)</t>
+          <t>38 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>204 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>409 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1229 (T)</t>
+          <t>1158 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2459 (T)</t>
+          <t>2317 (T)</t>
         </is>
       </c>
     </row>
@@ -2885,27 +2890,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>39 (T)</t>
+          <t>36 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>48 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>48 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>48 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>48 (E)</t>
+          <t>47 (E)</t>
         </is>
       </c>
     </row>
@@ -2917,27 +2922,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>39 (T)</t>
+          <t>36 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>195 (T)</t>
+          <t>181 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>391 (T)</t>
+          <t>362 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>485 (E)</t>
+          <t>471 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>485 (E)</t>
+          <t>471 (E)</t>
         </is>
       </c>
     </row>
@@ -2949,27 +2954,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>39 (T)</t>
+          <t>36 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>195 (T)</t>
+          <t>181 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>391 (T)</t>
+          <t>362 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1174 (T)</t>
+          <t>1086 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2349 (T)</t>
+          <t>2173 (T)</t>
         </is>
       </c>
     </row>
@@ -3054,27 +3059,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>37 (T)</t>
+          <t>33 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>44 (E)</t>
+          <t>43 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>44 (E)</t>
+          <t>43 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>44 (E)</t>
+          <t>43 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>44 (E)</t>
+          <t>43 (E)</t>
         </is>
       </c>
     </row>
@@ -3086,27 +3091,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>37 (T)</t>
+          <t>33 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>187 (T)</t>
+          <t>167 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>374 (T)</t>
+          <t>335 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>447 (E)</t>
+          <t>433 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>447 (E)</t>
+          <t>433 (E)</t>
         </is>
       </c>
     </row>
@@ -3118,27 +3123,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>37 (T)</t>
+          <t>33 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>187 (T)</t>
+          <t>167 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>374 (T)</t>
+          <t>335 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1122 (T)</t>
+          <t>1007 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2235 (E)</t>
+          <t>2015 (T)</t>
         </is>
       </c>
     </row>
@@ -3191,27 +3196,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>3 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>3 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>3 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>3 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4 (E)</t>
+          <t>3 (E)</t>
         </is>
       </c>
     </row>
@@ -3223,27 +3228,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>34 (T)</t>
+          <t>32 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>41 (E)</t>
+          <t>39 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>41 (E)</t>
+          <t>39 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>41 (E)</t>
+          <t>39 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>41 (E)</t>
+          <t>39 (E)</t>
         </is>
       </c>
     </row>
@@ -3255,27 +3260,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>34 (T)</t>
+          <t>32 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>173 (T)</t>
+          <t>161 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>347 (T)</t>
+          <t>322 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>417 (E)</t>
+          <t>393 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>417 (E)</t>
+          <t>393 (E)</t>
         </is>
       </c>
     </row>
@@ -3287,27 +3292,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>34 (T)</t>
+          <t>32 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>173 (T)</t>
+          <t>161 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>347 (T)</t>
+          <t>322 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1043 (T)</t>
+          <t>968 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2086 (E)</t>
+          <t>1937 (T)</t>
         </is>
       </c>
     </row>
@@ -3360,27 +3365,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1 (E)</t>
+          <t>5 (E)</t>
         </is>
       </c>
     </row>
@@ -3392,27 +3397,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12 (T)</t>
+          <t>40 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>17 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>17 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>17 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>17 (E)</t>
+          <t>52 (E)</t>
         </is>
       </c>
     </row>
@@ -3424,9 +3429,685 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>40 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>204 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>409 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>526 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>526 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>40 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>204 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>409 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1229 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2459 (T)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>39 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>48 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>39 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>195 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>391 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>485 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>485 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>39 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>195 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>391 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1174 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2349 (T)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>37 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>44 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>37 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>187 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>374 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>447 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>447 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>37 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>187 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>374 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1122 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2235 (E)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>34 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>41 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>34 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>173 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>347 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>417 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>417 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>34 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>173 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>347 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1043 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2086 (E)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>12 (T)</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>17 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12 (T)</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>62 (T)</t>
@@ -3439,12 +4120,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>172 (E)</t>
+          <t>175 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>172 (E)</t>
+          <t>175 (E)</t>
         </is>
       </c>
     </row>
@@ -3654,6 +4335,175 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T:1.00</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T:5.00</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T:10.00</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T:30.00</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>T:60.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E:0.12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E:1.25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>7 (T)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10 (E)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10 (E)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>10 (E)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E:12.50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>7 (T)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>35 (T)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>71 (T)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>101 (E)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>101 (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>E:62.50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>7 (T)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>35 (T)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>71 (T)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>214 (T)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>429 (T)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4036,27 +4886,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6 (E)</t>
+          <t>4 (E)</t>
         </is>
       </c>
     </row>
@@ -4068,27 +4918,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>28 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>42 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>42 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>42 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>66 (E)</t>
+          <t>42 (E)</t>
         </is>
       </c>
     </row>
@@ -4100,27 +4950,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>28 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>208 (T)</t>
+          <t>144 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>417 (T)</t>
+          <t>288 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>661 (E)</t>
+          <t>429 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>661 (E)</t>
+          <t>429 (E)</t>
         </is>
       </c>
     </row>
@@ -4132,27 +4982,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>41 (T)</t>
+          <t>28 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>208 (T)</t>
+          <t>144 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>417 (T)</t>
+          <t>288 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1251 (T)</t>
+          <t>866 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2502 (T)</t>
+          <t>1732 (T)</t>
         </is>
       </c>
     </row>
@@ -4242,22 +5092,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>65 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>65 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>65 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>65 (E)</t>
+          <t>66 (E)</t>
         </is>
       </c>
     </row>
@@ -4274,22 +5124,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>209 (T)</t>
+          <t>208 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>418 (T)</t>
+          <t>417 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>658 (E)</t>
+          <t>661 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>658 (E)</t>
+          <t>661 (E)</t>
         </is>
       </c>
     </row>
@@ -4306,22 +5156,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>209 (T)</t>
+          <t>208 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>418 (T)</t>
+          <t>417 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1255 (T)</t>
+          <t>1251 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2511 (T)</t>
+          <t>2502 (T)</t>
         </is>
       </c>
     </row>
@@ -4374,27 +5224,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5 (E)</t>
+          <t>6 (E)</t>
         </is>
       </c>
     </row>
@@ -4406,27 +5256,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>59 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>59 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>59 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>59 (E)</t>
+          <t>65 (E)</t>
         </is>
       </c>
     </row>
@@ -4438,27 +5288,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>193 (T)</t>
+          <t>209 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>386 (T)</t>
+          <t>418 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>594 (E)</t>
+          <t>658 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>594 (E)</t>
+          <t>658 (E)</t>
         </is>
       </c>
     </row>
@@ -4470,27 +5320,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>38 (T)</t>
+          <t>41 (T)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>193 (T)</t>
+          <t>209 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>386 (T)</t>
+          <t>418 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1160 (T)</t>
+          <t>1255 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2321 (T)</t>
+          <t>2511 (T)</t>
         </is>
       </c>
     </row>
@@ -4580,22 +5430,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>57 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>57 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>57 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>57 (E)</t>
+          <t>59 (E)</t>
         </is>
       </c>
     </row>
@@ -4612,22 +5462,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>190 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>381 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>570 (E)</t>
+          <t>594 (E)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>570 (E)</t>
+          <t>594 (E)</t>
         </is>
       </c>
     </row>
@@ -4644,22 +5494,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>190 (T)</t>
+          <t>193 (T)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>381 (T)</t>
+          <t>386 (T)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1143 (T)</t>
+          <t>1160 (T)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2286 (T)</t>
+          <t>2321 (T)</t>
         </is>
       </c>
     </row>

</xml_diff>